<commit_message>
feat: actualizar sistema a 18 concejales con DNI y asignaciones híbridas
</commit_message>
<xml_diff>
--- a/example (1).xlsx
+++ b/example (1).xlsx
@@ -623,7 +623,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -637,10 +637,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1880,26 +1876,27 @@
       </c>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="4" t="s">
+      <c r="A90" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="B90" s="4" t="s">
+      <c r="B90" s="2" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="4" t="s">
+      <c r="A91" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="B91" s="4" t="s">
+      <c r="B91" s="2" t="s">
         <v>171</v>
       </c>
+      <c r="C91" s="1"/>
     </row>
     <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="4" t="s">
+      <c r="A92" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="B92" s="4" t="s">
+      <c r="B92" s="2" t="s">
         <v>173</v>
       </c>
     </row>

</xml_diff>